<commit_message>
3 DECEMBER 2025 MORNING HOME
</commit_message>
<xml_diff>
--- a/NOVEMBER/NOVEMBER KITCHEN OUTSTANDING/NOVEMBER KSP OUTSTANDING.xlsx
+++ b/NOVEMBER/NOVEMBER KITCHEN OUTSTANDING/NOVEMBER KSP OUTSTANDING.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7500"/>
+    <workbookView windowWidth="28200" windowHeight="12620"/>
   </bookViews>
   <sheets>
     <sheet name="KSP (CHICKEN)" sheetId="1" r:id="rId1"/>
@@ -222,13 +222,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="7">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="dd\-mmm"/>
-    <numFmt numFmtId="180" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="180" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="181" formatCode="dd\-mmm"/>
+    <numFmt numFmtId="182" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -767,16 +767,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -916,80 +916,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1528,16 +1528,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8"/>
   <cols>
-    <col min="1" max="1" width="8.88571428571429" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.1428571428571" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.1428571428571" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.7238095238095" style="2" customWidth="1"/>
-    <col min="5" max="5" width="35.1238095238095" style="1" customWidth="1"/>
-    <col min="6" max="8" width="20.9904761904762" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.8571428571429" style="1"/>
-    <col min="10" max="16384" width="9.14285714285714" style="1"/>
+    <col min="1" max="1" width="8.8828125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="35.125" style="1" customWidth="1"/>
+    <col min="6" max="8" width="20.9921875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.859375" style="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="16" customHeight="1" spans="1:8">
@@ -1579,41 +1579,41 @@
       <c r="D2" s="7">
         <v>7.9</v>
       </c>
-      <c r="E2" s="8" t="str">
+      <c r="E2" s="14" t="str">
         <f>_xlfn.DISPIMG("ID_BC41213F5DF34C9FA380163A0DB01F5E",1)</f>
         <v>=DISPIMG("ID_BC41213F5DF34C9FA380163A0DB01F5E",1)</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="15">
         <v>48000</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="15">
         <f t="shared" ref="G2:G8" si="0">SUM(D2*F2)</f>
         <v>379200</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="16">
         <f>SUM(D2*F2+D3*F3)</f>
         <v>1118400</v>
       </c>
       <c r="L2" s="27"/>
     </row>
     <row r="3" s="1" customFormat="1" ht="64" customHeight="1" spans="1:11">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="12" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="10">
         <v>15.4</v>
       </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="9">
+      <c r="E3" s="17"/>
+      <c r="F3" s="15">
         <v>48000</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="15">
         <f t="shared" si="0"/>
         <v>739200</v>
       </c>
-      <c r="H3" s="15"/>
+      <c r="H3" s="18"/>
       <c r="K3" s="27"/>
     </row>
     <row r="4" s="1" customFormat="1" ht="43" customHeight="1" spans="1:11">
@@ -1623,67 +1623,67 @@
       <c r="B4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="10">
         <v>5.8</v>
       </c>
-      <c r="E4" s="8" t="str">
+      <c r="E4" s="14" t="str">
         <f>_xlfn.DISPIMG("ID_840C154ED5C648A3AFFBFA4A3E161E08",1)</f>
         <v>=DISPIMG("ID_840C154ED5C648A3AFFBFA4A3E161E08",1)</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="19">
         <v>48000</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="15">
         <f t="shared" si="0"/>
         <v>278400</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="16">
         <f>SUM(D4*F4+D5*F5+D6*F6)</f>
         <v>960600</v>
       </c>
       <c r="K4" s="27"/>
     </row>
     <row r="5" s="1" customFormat="1" ht="43" customHeight="1" spans="1:11">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="12" t="s">
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="10">
         <v>10.6</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="16">
+      <c r="E5" s="20"/>
+      <c r="F5" s="19">
         <v>48000</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="15">
         <f t="shared" si="0"/>
         <v>508800</v>
       </c>
-      <c r="H5" s="19"/>
+      <c r="H5" s="21"/>
       <c r="K5" s="27"/>
     </row>
     <row r="6" s="1" customFormat="1" ht="43" customHeight="1" spans="1:8">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="12" t="s">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="10">
         <v>5.1</v>
       </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="20">
+      <c r="E6" s="17"/>
+      <c r="F6" s="22">
         <v>34000</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="15">
         <f t="shared" si="0"/>
         <v>173400</v>
       </c>
-      <c r="H6" s="15"/>
+      <c r="H6" s="18"/>
     </row>
     <row r="7" s="1" customFormat="1" ht="43" customHeight="1" spans="1:8">
       <c r="A7" s="5">
@@ -1692,46 +1692,46 @@
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="10">
         <v>5.8</v>
       </c>
-      <c r="E7" s="8" t="str">
+      <c r="E7" s="14" t="str">
         <f>_xlfn.DISPIMG("ID_E04E53902D31429B9CCCC3BF0D548570",1)</f>
         <v>=DISPIMG("ID_E04E53902D31429B9CCCC3BF0D548570",1)</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="23">
         <v>48000</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="15">
         <f t="shared" si="0"/>
         <v>278400</v>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="24">
         <f t="shared" ref="H7:H11" si="1">SUM(G7:G8)</f>
         <v>782400</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="1" ht="65" customHeight="1" spans="1:8">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="21" t="s">
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="10">
         <v>10.5</v>
       </c>
-      <c r="E8" s="24"/>
-      <c r="F8" s="22">
+      <c r="E8" s="25"/>
+      <c r="F8" s="23">
         <v>48000</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="15">
         <f t="shared" si="0"/>
         <v>504000</v>
       </c>
-      <c r="H8" s="24"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" s="1" customFormat="1" ht="55" customHeight="1" spans="1:11">
       <c r="A9" s="5">
@@ -1740,47 +1740,47 @@
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="10">
         <v>4.85</v>
       </c>
-      <c r="E9" s="8" t="str">
+      <c r="E9" s="14" t="str">
         <f>_xlfn.DISPIMG("ID_D0D7F85949BC4377AA6D333D4CD41D95",1)</f>
         <v>=DISPIMG("ID_D0D7F85949BC4377AA6D333D4CD41D95",1)</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="22">
         <v>50000</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="22">
         <f t="shared" ref="G9:G12" si="2">D9*F9</f>
         <v>242500</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="24">
         <f t="shared" si="1"/>
         <v>1187250</v>
       </c>
       <c r="K9" s="27"/>
     </row>
     <row r="10" s="1" customFormat="1" ht="55" customHeight="1" spans="1:11">
-      <c r="A10" s="11"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="12" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="10">
         <v>18.895</v>
       </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="20">
+      <c r="E10" s="17"/>
+      <c r="F10" s="22">
         <v>50000</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="22">
         <f t="shared" si="2"/>
         <v>944750</v>
       </c>
-      <c r="H10" s="25"/>
+      <c r="H10" s="26"/>
       <c r="K10" s="27"/>
     </row>
     <row r="11" s="1" customFormat="1" ht="55" customHeight="1" spans="1:11">
@@ -1790,59 +1790,59 @@
       <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="10">
         <v>5.6</v>
       </c>
-      <c r="E11" s="8" t="str">
+      <c r="E11" s="14" t="str">
         <f>_xlfn.DISPIMG("ID_3B01175CA21E443B8591D01EA0BFD05B",1)</f>
         <v>=DISPIMG("ID_3B01175CA21E443B8591D01EA0BFD05B",1)</v>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="22">
         <v>52000</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="22">
         <f t="shared" si="2"/>
         <v>291200</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="24">
         <f t="shared" si="1"/>
         <v>1021200</v>
       </c>
       <c r="K11" s="27"/>
     </row>
     <row r="12" s="1" customFormat="1" ht="55" customHeight="1" spans="1:11">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="12" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="10">
         <v>14.6</v>
       </c>
-      <c r="E12" s="14"/>
-      <c r="F12" s="20">
+      <c r="E12" s="17"/>
+      <c r="F12" s="22">
         <v>50000</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="22">
         <f t="shared" si="2"/>
         <v>730000</v>
       </c>
-      <c r="H12" s="25"/>
+      <c r="H12" s="26"/>
       <c r="K12" s="27"/>
     </row>
-    <row r="13" s="1" customFormat="1" customHeight="1" spans="1:8">
-      <c r="A13" s="26"/>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20">
-        <f>SUM(H2:H11)</f>
+    <row r="13" s="1" customFormat="1" ht="15" customHeight="1" spans="1:8">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22">
+        <f>SUM(H2:H12)</f>
         <v>5069850</v>
       </c>
     </row>

</xml_diff>